<commit_message>
Plan B: columna Total (eje X + eje Y) y R1 verde hueco, R2 rojo sólido en la matriz de la plantilla
</commit_message>
<xml_diff>
--- a/deploy/plan_b/Plantilla_Horizontes_Shot_Nutresa.xlsx
+++ b/deploy/plan_b/Plantilla_Horizontes_Shot_Nutresa.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -87,6 +87,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -177,7 +178,13 @@
             <v>Fijos</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="9AA5B4"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+              <a:solidFill>
+                <a:srgbClr val="9AA5B4"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -204,7 +211,11 @@
             <v>INSUMEX R1</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+              <a:solidFill>
+                <a:srgbClr val="1F7A3A"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -231,7 +242,13 @@
             <v>INSUMEX R2</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="C62828"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+              <a:solidFill>
+                <a:srgbClr val="C62828"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -258,7 +275,11 @@
             <v>NUTRIWHAT R1</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+              <a:solidFill>
+                <a:srgbClr val="1F7A3A"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -285,7 +306,13 @@
             <v>NUTRIWHAT R2</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="C62828"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+              <a:solidFill>
+                <a:srgbClr val="C62828"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -695,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -742,22 +769,29 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>4. La hoja Matriz muestra los 8 fijos y los 2 vivos en R1 y R2. Proyéctala.</t>
+          <t>4. La hoja Matriz muestra los 8 fijos y los 2 vivos en R1 (verde, hueco) y R2 (rojo, sólido). Proyéctala.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>5. Para conversar con la sala usa los 6 criterios y la columna Total (eje X + eje Y). T2M, Eje X y Eje Y solo ubican la burbuja en la matriz.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Si ya tienes los promedios por criterio (por ejemplo, contados a mano), escríbelos en Resultados, filas "Promedio digitado", y deja vacía la hoja Votos.</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Si ya tienes los promedios por criterio (por ejemplo, contados a mano), escríbelos en Resultados, filas "Promedio digitado", y deja vacía la hoja Votos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Nunca escribas nombres en la hoja Votos: la papeleta es anónima.</t>
         </is>
@@ -861,7 +895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -877,6 +911,7 @@
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1048,6 +1083,11 @@
           <t>TAM</t>
         </is>
       </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1101,6 +1141,10 @@
       <c r="M15" t="n">
         <v>5</v>
       </c>
+      <c r="N15" s="7">
+        <f>IF(OR(ISNA(K15),ISNA(L15)),NA(),K15+L15)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1154,6 +1198,10 @@
       <c r="M16" t="n">
         <v>6</v>
       </c>
+      <c r="N16" s="7">
+        <f>IF(OR(ISNA(K16),ISNA(L16)),NA(),K16+L16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1207,6 +1255,10 @@
       <c r="M17" t="n">
         <v>5</v>
       </c>
+      <c r="N17" s="7">
+        <f>IF(OR(ISNA(K17),ISNA(L17)),NA(),K17+L17)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1260,6 +1312,10 @@
       <c r="M18" t="n">
         <v>6</v>
       </c>
+      <c r="N18" s="7">
+        <f>IF(OR(ISNA(K18),ISNA(L18)),NA(),K18+L18)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -1277,12 +1333,12 @@
           <t>INSUMEX</t>
         </is>
       </c>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
-      <c r="I22" s="7" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="n"/>
+      <c r="H22" s="8" t="n"/>
+      <c r="I22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1293,12 +1349,12 @@
           <t>NUTRIWHAT</t>
         </is>
       </c>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-      <c r="H23" s="7" t="n"/>
-      <c r="I23" s="7" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="8" t="n"/>
+      <c r="F23" s="8" t="n"/>
+      <c r="G23" s="8" t="n"/>
+      <c r="H23" s="8" t="n"/>
+      <c r="I23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1309,12 +1365,12 @@
           <t>INSUMEX</t>
         </is>
       </c>
-      <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
-      <c r="F24" s="7" t="n"/>
-      <c r="G24" s="7" t="n"/>
-      <c r="H24" s="7" t="n"/>
-      <c r="I24" s="7" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="8" t="n"/>
+      <c r="H24" s="8" t="n"/>
+      <c r="I24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1325,12 +1381,12 @@
           <t>NUTRIWHAT</t>
         </is>
       </c>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
-      <c r="F25" s="7" t="n"/>
-      <c r="G25" s="7" t="n"/>
-      <c r="H25" s="7" t="n"/>
-      <c r="I25" s="7" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="8" t="n"/>
+      <c r="H25" s="8" t="n"/>
+      <c r="I25" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -1397,6 +1453,11 @@
           <t>TAM</t>
         </is>
       </c>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
@@ -1437,6 +1498,10 @@
       <c r="M29" t="n">
         <v>10</v>
       </c>
+      <c r="N29" s="6">
+        <f>K29+L29</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="B30" t="inlineStr">
@@ -1477,6 +1542,10 @@
       <c r="M30" t="n">
         <v>6</v>
       </c>
+      <c r="N30" s="6">
+        <f>K30+L30</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
@@ -1517,6 +1586,10 @@
       <c r="M31" t="n">
         <v>7</v>
       </c>
+      <c r="N31" s="6">
+        <f>K31+L31</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="B32" t="inlineStr">
@@ -1557,6 +1630,10 @@
       <c r="M32" t="n">
         <v>4</v>
       </c>
+      <c r="N32" s="6">
+        <f>K32+L32</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="B33" t="inlineStr">
@@ -1597,6 +1674,10 @@
       <c r="M33" t="n">
         <v>2</v>
       </c>
+      <c r="N33" s="6">
+        <f>K33+L33</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="B34" t="inlineStr">
@@ -1637,6 +1718,10 @@
       <c r="M34" t="n">
         <v>1</v>
       </c>
+      <c r="N34" s="6">
+        <f>K34+L34</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="B35" t="inlineStr">
@@ -1677,6 +1762,10 @@
       <c r="M35" t="n">
         <v>1</v>
       </c>
+      <c r="N35" s="6">
+        <f>K35+L35</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="B36" t="inlineStr">
@@ -1716,6 +1805,10 @@
       </c>
       <c r="M36" t="n">
         <v>8</v>
+      </c>
+      <c r="N36" s="6">
+        <f>K36+L36</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1742,7 +1835,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Fijos en gris; cada vivo aparece en R1 y R2. Tamaño de la burbuja: TAM. Horizontes: H1 hasta radio 4,5; H2 hasta 9; H3 afuera.</t>
+          <t>Fijos en gris; cada vivo aparece en R1 (verde, hueco) y R2 (rojo, sólido). Tamaño de la burbuja: TAM. Horizontes: H1 hasta radio 4,5; H2 hasta 9; H3 afuera.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[T4] Plan B: columna Total (eje X + eje Y) y R1 verde hueco, R2 rojo sólido en la matriz de la plantilla
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deploy/plan_b/Plantilla_Horizontes_Shot_Nutresa.xlsx
+++ b/deploy/plan_b/Plantilla_Horizontes_Shot_Nutresa.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -87,6 +87,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -177,7 +178,13 @@
             <v>Fijos</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="9AA5B4"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+              <a:solidFill>
+                <a:srgbClr val="9AA5B4"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -204,7 +211,11 @@
             <v>INSUMEX R1</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+              <a:solidFill>
+                <a:srgbClr val="1F7A3A"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -231,7 +242,13 @@
             <v>INSUMEX R2</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="C62828"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+              <a:solidFill>
+                <a:srgbClr val="C62828"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -258,7 +275,11 @@
             <v>NUTRIWHAT R1</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+              <a:solidFill>
+                <a:srgbClr val="1F7A3A"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -285,7 +306,13 @@
             <v>NUTRIWHAT R2</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="C62828"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+              <a:solidFill>
+                <a:srgbClr val="C62828"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -695,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -742,22 +769,29 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>4. La hoja Matriz muestra los 8 fijos y los 2 vivos en R1 y R2. Proyéctala.</t>
+          <t>4. La hoja Matriz muestra los 8 fijos y los 2 vivos en R1 (verde, hueco) y R2 (rojo, sólido). Proyéctala.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>5. Para conversar con la sala usa los 6 criterios y la columna Total (eje X + eje Y). T2M, Eje X y Eje Y solo ubican la burbuja en la matriz.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Si ya tienes los promedios por criterio (por ejemplo, contados a mano), escríbelos en Resultados, filas "Promedio digitado", y deja vacía la hoja Votos.</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Si ya tienes los promedios por criterio (por ejemplo, contados a mano), escríbelos en Resultados, filas "Promedio digitado", y deja vacía la hoja Votos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Nunca escribas nombres en la hoja Votos: la papeleta es anónima.</t>
         </is>
@@ -861,7 +895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -877,6 +911,7 @@
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1048,6 +1083,11 @@
           <t>TAM</t>
         </is>
       </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1101,6 +1141,10 @@
       <c r="M15" t="n">
         <v>5</v>
       </c>
+      <c r="N15" s="7">
+        <f>IF(OR(ISNA(K15),ISNA(L15)),NA(),K15+L15)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1154,6 +1198,10 @@
       <c r="M16" t="n">
         <v>6</v>
       </c>
+      <c r="N16" s="7">
+        <f>IF(OR(ISNA(K16),ISNA(L16)),NA(),K16+L16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1207,6 +1255,10 @@
       <c r="M17" t="n">
         <v>5</v>
       </c>
+      <c r="N17" s="7">
+        <f>IF(OR(ISNA(K17),ISNA(L17)),NA(),K17+L17)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1260,6 +1312,10 @@
       <c r="M18" t="n">
         <v>6</v>
       </c>
+      <c r="N18" s="7">
+        <f>IF(OR(ISNA(K18),ISNA(L18)),NA(),K18+L18)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -1277,12 +1333,12 @@
           <t>INSUMEX</t>
         </is>
       </c>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
-      <c r="I22" s="7" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="n"/>
+      <c r="H22" s="8" t="n"/>
+      <c r="I22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1293,12 +1349,12 @@
           <t>NUTRIWHAT</t>
         </is>
       </c>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-      <c r="H23" s="7" t="n"/>
-      <c r="I23" s="7" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="8" t="n"/>
+      <c r="F23" s="8" t="n"/>
+      <c r="G23" s="8" t="n"/>
+      <c r="H23" s="8" t="n"/>
+      <c r="I23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1309,12 +1365,12 @@
           <t>INSUMEX</t>
         </is>
       </c>
-      <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
-      <c r="F24" s="7" t="n"/>
-      <c r="G24" s="7" t="n"/>
-      <c r="H24" s="7" t="n"/>
-      <c r="I24" s="7" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="8" t="n"/>
+      <c r="H24" s="8" t="n"/>
+      <c r="I24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1325,12 +1381,12 @@
           <t>NUTRIWHAT</t>
         </is>
       </c>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
-      <c r="F25" s="7" t="n"/>
-      <c r="G25" s="7" t="n"/>
-      <c r="H25" s="7" t="n"/>
-      <c r="I25" s="7" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="8" t="n"/>
+      <c r="H25" s="8" t="n"/>
+      <c r="I25" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -1397,6 +1453,11 @@
           <t>TAM</t>
         </is>
       </c>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
@@ -1437,6 +1498,10 @@
       <c r="M29" t="n">
         <v>10</v>
       </c>
+      <c r="N29" s="6">
+        <f>K29+L29</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="B30" t="inlineStr">
@@ -1477,6 +1542,10 @@
       <c r="M30" t="n">
         <v>6</v>
       </c>
+      <c r="N30" s="6">
+        <f>K30+L30</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
@@ -1517,6 +1586,10 @@
       <c r="M31" t="n">
         <v>7</v>
       </c>
+      <c r="N31" s="6">
+        <f>K31+L31</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="B32" t="inlineStr">
@@ -1557,6 +1630,10 @@
       <c r="M32" t="n">
         <v>4</v>
       </c>
+      <c r="N32" s="6">
+        <f>K32+L32</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="B33" t="inlineStr">
@@ -1597,6 +1674,10 @@
       <c r="M33" t="n">
         <v>2</v>
       </c>
+      <c r="N33" s="6">
+        <f>K33+L33</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="B34" t="inlineStr">
@@ -1637,6 +1718,10 @@
       <c r="M34" t="n">
         <v>1</v>
       </c>
+      <c r="N34" s="6">
+        <f>K34+L34</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="B35" t="inlineStr">
@@ -1677,6 +1762,10 @@
       <c r="M35" t="n">
         <v>1</v>
       </c>
+      <c r="N35" s="6">
+        <f>K35+L35</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="B36" t="inlineStr">
@@ -1716,6 +1805,10 @@
       </c>
       <c r="M36" t="n">
         <v>8</v>
+      </c>
+      <c r="N36" s="6">
+        <f>K36+L36</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1742,7 +1835,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Fijos en gris; cada vivo aparece en R1 y R2. Tamaño de la burbuja: TAM. Horizontes: H1 hasta radio 4,5; H2 hasta 9; H3 afuera.</t>
+          <t>Fijos en gris; cada vivo aparece en R1 (verde, hueco) y R2 (rojo, sólido). Tamaño de la burbuja: TAM. Horizontes: H1 hasta radio 4,5; H2 hasta 9; H3 afuera.</t>
         </is>
       </c>
     </row>

</xml_diff>